<commit_message>
Weekly briefing 2026-05-01 to 2026-05-07
https://claude.ai/code/session_018DaKXaeq9PyJfpQTAwb6qs
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,6 +768,356 @@
         <v>2</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CFPB Final Rule: Revised Section 1071 Small Business Lending Data Collection</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CFPB published a substantially revised Section 1071 small business lending data rule in the Federal Register. Coverage applies to lenders with 1,000+ covered small business originations in each of the two prior years; Farm Credit System lenders are excluded. Compliance date is January 1, 2028 (first SBLR filing June 1, 2029). Rule effective June 30, 2026. Bureau signals good-faith supervisory grace period for initial collection year.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/05/01/2026-08494/small-business-lending-under-the-equal-credit-opportunity-act-regulation-b</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CFPB</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NCUA Announces Eleventh Round of Deregulation Proposals</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NCUA proposed two rules: (1) raise the DIMIA major assets prohibition threshold from $2.5B to $10B; (2) streamline Part 741 share insurance regulations for FISCUs by removing duplicative cross-references. Part of NCUA's ongoing Deregulation Project; Federal Register notice for share insurance published May 7, 2026.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://ncua.gov/newsroom/press-release/2026/ncua-announces-eleventh-round-deregulation-proposals</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FinCEN Issues Consolidated and Updated CDD FAQs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FinCEN consolidated three prior CDD FAQ sets into one document and updated answers to align with the February 13, 2026 Account Opening Exceptive Relief Order (FIN-2026-R001). Beneficial ownership verification shifts to a relationship-based model — only required at first account opening or upon flagged changes. Adoption of the exceptive relief remains at each institution's discretion.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.fincen.gov/resources/statutes-and-regulations/cdd-rule-faqs</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FinCEN</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>California DFPI Monthly Bulletin: Digital Financial Assets Law License Deadline Approaching (July 1, 2026)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DFPI's May 2026 Monthly Bulletin reminds covered entities that by July 1, 2026, anyone offering digital-asset activities (crypto exchanges, custodians, kiosks) for California residents must hold a DFAL license or qualify for an exemption. State-chartered banks and CUs with crypto programs should confirm their status. Bulletin also notes DFPI's first administrative CCFPL decision affirming jurisdiction over debt-settlement services.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://dfpi.ca.gov/news/monthly-bulletins/monthly-bulletin-may-2026/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CA DFPI</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Federal Banking Agencies Issue Annual Host State Loan-to-Deposit Ratios</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Federal Reserve, FDIC, and OCC jointly released the 2026 annual host state loan-to-deposit ratios as required under the Riegle-Neal Act, replacing 2025 ratios. Banks use these to verify compliance with the prohibition on acquiring interstate branches primarily to gather out-of-state deposits.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/bcreg20260501a.htm</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Federal Reserve / FDIC / OCC</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Federal Reserve Vice Chair Bowman Speech: Artificial Intelligence in the Financial System</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Vice Chair Bowman addressed the FSOC AI Roundtable on Cybersecurity. She noted the Fed, OCC, and FDIC recently amended model risk management guidance to clarify it does not apply to generative or agentic AI. Raised cybersecurity concerns about dual-use AI capable of identifying system vulnerabilities. No new rulemaking announced.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/speech/bowman20260501a.htm</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Federal Reserve Vice Chair Bowman Speech: Consumer Fraud Protection</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Vice Chair Bowman spoke at the 2026 Women in Housing and Finance Symposium on consumer fraud, including authorized push payment fraud. No new rulemaking or guidance announced; reflects ongoing supervisory attention to banks' fraud-prevention programs.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/speech/bowman20260505a.htm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FDIC Issues Monthly List of Banks Examined for CRA Compliance</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Routine FDIC monthly release listing state nonmember banks evaluated for Community Reinvestment Act compliance, covering examination ratings assigned in the most recent reporting period.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/press-releases/2026/fdic-issues-list-banks-examined-cra-compliance-3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>OCC Releases CRA Performance Evaluations for 21 National Banks and FSAs</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OCC released CRA performance evaluations that became public April 1–30, 2026, covering 21 national banks and federal savings associations. Full evaluation reports are available on the OCC website.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-34.html</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>New York DFS and Comptroller Designate Banking Development District (Shandaken/Olive)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NY Comptroller DiNapoli and DFS Acting Superintendent Asrow approved the 59th BDD designation for towns of Shandaken and Olive (Ulster County), with a $10M state deposit at Ulster Savings Bank. BDD program incentivizes bank and credit union branches in underserved communities.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.dfs.ny.gov/reports_and_publications/press_releases/pr20260506</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NY DFS</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-05-08 to 2026-05-14
8 items: Fed Chair transition (Miran resignation/Warsh confirmation), FDIC Spring 2023 bank-run study, Fed discount window survey results, Illinois IDFPR complaint portal, Fed enforcement terminations, Columbia Financial merger approval, OCC criminal offenses report, Bowman community banking speech.
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1118,6 +1118,286 @@
         <v>2</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Federal Reserve Governor Miran Resigns; Kevin Warsh Confirmed as Incoming Chair</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Governor Stephen Miran submitted his resignation effective when or shortly before incoming Chair Kevin Warsh is sworn in. The Senate confirmed Warsh as both a Board member and Chairman earlier in the week. Miran dissented at every FOMC meeting since joining the Board in September 2025. Warsh's leadership is expected to reshape the Fed's monetary policy and supervisory agenda; banks should watch for early signals on capital framework, stress-testing, and resolution-planning requirements.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/other20260514b.htm</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FDIC Releases Staff Study on Deposit Flight at Spring 2023 Failed Banks (SVB, Signature, First Republic)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>"Dissecting Depositor Flight" uses transaction-level data to show that depositor size and sophistication are the primary run-risk predictors. The top 0.5% of depositors controlled 62% of Signature's deposits and 50% of First Republic's. Uninsured balances were 94% at SVB, 76% at Signature, and 74% at First Republic. SVB and Signature each lost more than half their deposits in 10 days. Will inform supervisory expectations on uninsured deposit concentration and liquidity stress testing.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/press-releases/2026/fdic-releases-staff-study-deposit-flows-three-failed-banks-spring-2023</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Federal Reserve Releases Senior Financial Officers Survey Results on Discount Window and Reserve Management</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Results from two surveys (Jan-Feb and March 2026) of senior financial officers covering banks' views on discount window operating days and reserve balance management. Survey 1 targeted banks with median assets under $5 billion; Survey 2 covered banks holding ~75% of system reserves. Results provide transparency on liquidity cushion practices and use of Fed facilities across institution sizes.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/other20260514a.htm</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Illinois IDFPR Launches Unified Online Consumer Complaint Portal for Banks and Financial Institutions</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>IDFPR launched a new online portal accepting complaints for both the Division of Banking (DOB) and Division of Financial Institutions (DFI) — the first unified interface for both divisions. Creates a more accessible consumer complaint intake process. State-chartered banks and financial institutions supervised by IDFPR should brief compliance teams on the new channel, which may increase complaint volume and speed of regulatory notification.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://idfpr.illinois.gov/news/2026/idfpr-launches-new-online-portal-streamline-consumer-financial-complaints.html</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Illinois</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Illinois IDFPR</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Federal Reserve Terminates Written Agreements with F&amp;M Holding Company and Thread Bancorp</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The Fed terminated 15+ year-old written agreements with F&amp;M Holding Company, Inc. (Manchester, GA; agreement from May 2011) and Thread Bancorp, Inc. (Rogersville, TN; agreement from May 2010). Both institutions have returned to satisfactory supervisory condition.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/enforcement20260512a.htm</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Federal Reserve Approves Columbia Financial's Acquisition of Northfield Bancorp (Columbia Bank MHC Conversion)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The Federal Reserve approved Columbia Bank MHC and Columbia Financial, Inc. (Fair Lawn, NJ) applications for mutual-to-stock conversion and simultaneous acquisition of Northfield Bancorp. The OCC approved the Bank Merger Act application on May 4, 2026. Combined institution will be a larger NJ-chartered commercial bank.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/orders20260508a.htm</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>OCC Issues Report Identifying Criminal Regulatory Offenses Under Executive Order 14294</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>In compliance with EO 14294 ("Fighting Overcriminalization in Federal Statutes"), the OCC published a report listing all criminal regulatory offenses within its jurisdiction, penalty ranges, and required mental-state standards. Outlines the OCC's framework for DOJ referrals of potential criminal violations. Relevant for compliance officers building internal escalation protocols.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.occ.treas.gov/news-issuances/news-releases/2026/nr-occ-2026-36.html</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Vice Chair Bowman Delivers Opening Remarks at Kansas City Fed's 2026 Future of Banking Conference</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Vice Chair for Supervision Bowman delivered pre-recorded opening remarks for community bankers, signaling continued commitment to tailored, risk-based supervision and deregulatory agenda for community institutions ahead of the Chair transition. No new rules announced.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/speech/bowman20260514a.htm</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-05-15 to 2026-05-21
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1398,6 +1398,356 @@
         <v>2</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>FFIEC Proposes First Revision to CAMELS Rating System Since 1996</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FFIEC invited public comment on the first comprehensive revision to the Uniform Financial Institutions Rating System (CAMELS) in 30 years. Proposal retains the six-component structure but refocuses ratings on material financial risks and quantitative factors, shifting away from process-heavy supervision. Applies to all FFIEC-supervised banks and credit unions. Comments due August 17, 2026.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.ffiec.gov/news/press-releases/2026/pr-05-19</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>FFIEC</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>OCC Issues Two Final Rules: Preemption of State Interest-on-Escrow Laws</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OCC finalized two rules (effective June 18, 2026) confirming national banks may decide whether to pay interest on mortgage escrow accounts, and formally preempting state laws in 14 jurisdictions (CA, CT, ME, MD, MA, MN, NY, OR, RI, UT, VT, WI, Guam, USVI) that mandate such interest payments.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://occ.gov/news-issuances/news-releases/2026/nr-occ-2026-37.html</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NCUA Proposes Rule for Permitted Payment Stablecoin Issuer Standards</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>NCUA issued an NPRM establishing operational and risk-management standards for credit unions seeking NCUA-licensed Permitted Payment Stablecoin Issuer (PPSI) status under the GENIUS Act. Standards align with those proposed for bank subsidiaries and cover capital, liquidity, AML/CFT, and reserve requirements. Comment period closes July 17, 2026.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://ncua.gov/newsroom/press-release/2026/ncua-announces-proposed-rule-permitted-payment-stablecoin-issuer-standards</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Federal Reserve Requests Comment on Payment Account Proposal</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fed proposed a new 'payment account' at Reserve Banks for eligible financial institutions to use solely for clearing and settling their own payments. Accounts are fully prefunded, capped at the lesser of $500M or 10% of total assets, and may not be used for correspondent banking or settling third-party payments.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/other20260520a.htm</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>OCC Advances Priority of Reducing Regulatory Burden for Community Banks</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OCC published deregulatory actions for community banks: effective January 1, 2026 guidance removed mandatory exam activities for CRA, fair lending, derivatives, and trading; examiners now tailor reviews to each bank's activities and material financial risks. OCC also updated CRA exam scheduling with greater frequency discretion.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-38.html</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Federal Reserve Terminates Cease-and-Desist Orders Against UBS and Credit Suisse (Archegos)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Fed terminated July 2023 cease-and-desist orders against UBS Group AG, Credit Suisse AG, Credit Suisse Holdings (USA), and Credit Suisse AG (New York Branch) for unsafe counterparty credit-risk practices tied to Archegos Capital Management, effective May 12, 2026, following remediation and payment of ~$268.5M in civil penalties.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/enforcement20260515a.htm</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>OCC Announces May 2026 Enforcement Actions</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>OCC released May 2026 enforcement actions including a Consent Order against Community Federal Savings Bank (Woodhaven, NY) for BSA/AML compliance program deficiencies, and an Order Terminating the Formal Agreement with First National Bank of Williamson (Williamson, WV).</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-40.html</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FDIC FIL-22-2026: Updated Q&amp;As on Official Signs and Advertising Requirements</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FDIC issued updated Q&amp;As implementing its January 2026 Part 328 amendments on digital FDIC signage for websites, mobile apps, and ATMs. Q&amp;As address specific implementation questions from banks, trade groups, and technology vendors to support compliance readiness.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/financial-institution-letters/2026/updated-questions-and-answers-regarding-fdic-official-signs</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>California DFPI Orders Hermes Bitcoin to Cease All California Bitcoin ATM Operations</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>California DFPI settlement required Anh Management LLC (d/b/a Hermes Bitcoin), operator of 42 Bitcoin ATMs across Southern California, to cease all digital financial asset business in California by May 20, 2026. Alleged violations: exceeding DFAL's $1,000/day cash cap, failure to verify customer identity, and AML non-compliance. Suspended $9.9M penalty becomes due upon non-compliance.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://dfpi.ca.gov/news/monthly-bulletins/monthly-bulletin-may-2026/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>California DFPI</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Federal Reserve Names Powell Chair Pro Tempore Pending Warsh Swearing-In</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fed Board named Jerome H. Powell as chair pro tempore upon expiration of his term, pending swearing-in of Kevin M. Warsh. Vice Chair Bowman and Governor Miran issued a statement supporting the designation. No immediate change to Fed regulatory or monetary policy is anticipated during the transition.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/other20260515a.htm</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-05-22 to 2026-05-28
8 items: two Trump executive orders (fintech innovation, financial-integrity/CDD),
FDIC GENIUS Act BSA/sanctions stablecoin NPRM, Fed Regulation A NPRM, GSIB
resolution plan feedback letters, OCC abstention statement, Warsh oath of
office, FHFA Q1 2026 HPI.
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,6 +1748,286 @@
         <v>3</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Executive Order: Restoring Integrity to America's Financial System</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>President Trump signed an EO directing Treasury to issue a BSA red-flag advisory for immigration-related financial activity and mandating CDD/CIP rule revisions within 60–180 days. CFPB must consider deportation as an ability-to-repay risk factor within 60 days. All banks and credit unions face potential BSA program amendments via forthcoming rulemaking.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/05/22/2026-10400/restoring-integrity-to-americas-financial-system</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>White House / Treasury</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Executive Order: Integrating Financial Technology Innovation into Regulatory Frameworks</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Directs each federal financial regulator to conduct a 90-day review of barriers to bank-fintech partnerships and application processes for fintech charters. The Federal Reserve must evaluate within 120 days whether non-bank fintechs and digital asset firms should obtain direct Fed payment account access. Regulatory guidance and rule changes expected over next 90–120 days.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/05/22/2026-10399/integrating-financial-technology-innovation-into-regulatory-frameworks</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>White House / Multiple Agencies</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FDIC NPRM: BSA/Sanctions Compliance Standards for FDIC-Supervised Permitted Payment Stablecoin Issuers (GENIUS Act)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The FDIC Board approved a proposed rule requiring FDIC-supervised permitted payment stablecoin issuers to establish BSA/AML/CFT and OFAC sanctions compliance programs. Third GENIUS Act rulemaking at the FDIC, following December 2025 application procedures and April 2026 prudential standards rules. Banks contemplating stablecoin issuance must track and comment.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/press-releases/2026/fdic-board-approves-proposal-address-bank-secrecy-act-and-sanctions</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Federal Reserve NPRM: Regulation A Amendments — Discount Window Credit Restrictions for Payment Account Holders</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The Fed proposed amending Regulation A to prohibit Reserve Banks from extending discount window credit to Payment Account holders, ring-fencing traditional discount window access away from non-bank entities that may obtain Fed master accounts under the companion Payment Account proposal. Comment period closes July 27, 2026.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/05/26/2026-10376/regulation-a-extensions-of-credit-by-federal-reserve-banks</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Fed and FDIC Publish Resolution Plan Feedback Letters for 8 GSIBs and 56 Foreign Banking Organizations</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The Federal Reserve and FDIC jointly published feedback letters on July 2025 resolution plans submitted by the eight U.S. GSIBs and 56 foreign banking organizations. No shortcomings or deficiencies were identified. Derivatives-related weaknesses from 2023 plans for four GSIBs were confirmed as resolved. OCC Comptroller abstained from the FDIC vote, citing structural concerns with the resolution planning regime.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/bcreg20260522a.htm</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Federal Reserve / FDIC</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>OCC Comptroller Issues Statement on Abstention from FDIC Resolution Plan Vote</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Comptroller Gould explained his abstention from the FDIC's resolution plan feedback vote, citing unresolved legal and conceptual deficiencies in the current process and its limited supervisory value. Signals continued OCC skepticism and potential advocacy for legislative or regulatory reform of Title I/II resolution planning requirements.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-41.html</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Kevin Warsh Sworn in as Federal Reserve Chair</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Kevin Warsh took the oath of office at the White House on May 22, 2026, becoming the 11th Fed chair of the modern era. He succeeds Jerome Powell, who remains as a governor. Warsh has signaled a reform-oriented agenda including regulatory burden reduction, capital rule modernization, and a reassessment of supervisory posture.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/other20260522a.htm</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>FHFA Q1 2026 House Price Index: U.S. Home Prices +1.7% Year-Over-Year</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FHFA released Q1 2026 HPI data showing U.S. home prices rose 1.7% year-over-year and 0.5% quarter-over-quarter. Prices rose in 42 states; Illinois led at +7.3%. Relevant to residential mortgage collateral valuations and CRA performance context; no direct compliance obligation.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.fhfa.gov/news/news-release/u.s.-house-prices-rise-1.7-percent-year-over-year-up-0.5-percent-quarter-over-quarter</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>FHFA</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-05-29 to 2026-06-04
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2028,6 +2028,216 @@
         <v>2</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Agencies Remove Additional References to Reputation Risk in 15 Interagency Documents</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>The Federal Reserve, OCC, and FDIC jointly reissued 15 interagency supervisory guidance documents with all reputation-risk references removed, following their April 2026 final rule abolishing the concept. Updated documents cover asset securitization, subprime lending, BOLI, CIP FAQs, home equity, remote deposit capture, counterparty credit risk, cyber-incident statements (ATM attacks, DDoS, cyber insurance, cyber extortion), operational resilience, elder financial exploitation, and loan participations. Effective immediately; all banks should verify their exam-prep and compliance materials align with the revised guidance.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/bcreg20260602a.htm</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Federal Reserve / OCC / FDIC</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SEC Proposes Rescission of Climate-Related Disclosure Rules</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>The SEC voted to propose full rescission of the March 2024 climate-related disclosure rules (Release No. 33-11275), arguing they exceed statutory authority and conflict with a materiality-based approach. Would eliminate Scope 1/2/3 GHG, climate-risk scenario, and related disclosures for all public companies including bank holding companies. 60-day public comment period following Federal Register publication.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/newsroom/press-releases/2026-49-sec-proposes-rescission-climate-related-disclosure-rules</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FHA Request for Information: Modernization of Single Family Minimum Property Requirements (MPR)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>HUD/FHA published a Request for Information (Docket No. FR-6609-N-01) in the Federal Register seeking public feedback on modernizing its Minimum Property Requirements for FHA-insured single-family homes. FHA aims to balance collateral-risk management with reducing homeownership access barriers. FHA-approved lenders and mortgage originators should review and consider filing comments. Comment deadline: June 29, 2026.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/05/29/2026-10766/request-for-information-regarding-single-family-minimum-property-requirements-mpr</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>HUD / FHA</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>FDIC Publishes April 2026 Enforcement Actions</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FDIC released April 2026 enforcement actions including two Flood Disaster Protection Act violations (failure to provide timely flood-insurance notice; failure to force-place flood insurance in 20 loan cases) and an informal AML/CFT agreement with a bank for deficiencies in risk assessment, CDD, SAR, CTR procedures, and absence of a qualified AML officer and training program.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/press-releases/2026/fdic-publishes-april-enforcement-actions</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Prudential Bank Regulators Testify Before House Financial Services Committee on Oversight</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Fed Vice Chair Bowman, Comptroller Gould, FDIC Chair Hill, and Acting NCUA Chair Hauptman testified at a House Financial Services Committee oversight hearing. Regulators highlighted deregulatory agendas: right-sizing capital requirements, refocusing exams on material financial risk, and building stablecoin/AI supervisory frameworks. Bowman noted AI has accelerated identification of cyber vulnerabilities. No binding rule resulted.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.fdic.gov/news/speeches/2026/oversight-prudential-regulators</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Federal Reserve / OCC / FDIC / NCUA</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Texas DOB Issues Consent Order Against Individual Banker (Kelsi Marie Karr)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>The Texas Banking Commissioner issued a Consent Order on June 1, 2026 prohibiting Kelsi Marie Karr from further participation in banking activities in Texas. This is a narrow individual-prohibition order and does not directly affect any chartered institution.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.dob.texas.gov/news-and-events/press-releases</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Texas Department of Banking</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-06-05 to 2026-06-11
https://claude.ai/code/session_01MYDtUpKGry6QpiMNczsuik
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2238,6 +2238,321 @@
         <v>2</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Financial Data Transparency Act: Joint Data Standards Final Rule</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Nine federal financial regulators (Fed, FDIC, OCC, CFPB, SEC, FHFA, NCUA, CFTC, Treasury) jointly published a final rule implementing mandatory data standards under the Financial Data Transparency Act of 2022, requiring common identifiers (LEI, ISO dates, machine-readable schemas) for all regulatory data submissions. Effective October 1, 2026.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/bulletins/2026/bulletin-2026-25.html</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Fed / FDIC / OCC / CFPB / SEC / FHFA / NCUA / CFTC / Treasury</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>NCUA Interim Final Rule: Federal Credit Union Non-Interest Charges and Fees (State Law Preemption)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NCUA published an interim final rule asserting exclusive federal authority over FCU non-interest charges and fees, including interchange fees, preempting state laws such as Illinois' Interchange Fee Prohibition Act. Mirrors OCC's earlier action for national banks. Effective June 30, 2026; comments due July 9, 2026.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/06/09/2026-11559/preemption-federal-credit-union-non-interest-charges-and-fees</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Oregon HB 4116: DIDMCA Opt-Out — Consumer Loan Interest Rate Cap Effective June 5</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Oregon's opt-out of DIDMCA Section 521 became effective June 5, 2026, barring out-of-state FDIC-insured state-chartered banks from charging above Oregon's 36% APR cap on consumer finance loans of $50,000 or less to Oregon borrowers. Signed April 7 by Governor Kotek. Requires immediate compliance review for interstate consumer lenders operating in Oregon.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://oregonbusinessreport.com/2026/06/new-law-protects-consumers-from-predatory-high-interest-loans/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Oregon</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Oregon Legislature</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>CFPB Statement: Ability to Repay and Immigration Status</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CFPB published a Federal Register statement under EO 14406 reminding creditors that ATR requirements under TILA/Reg Z may require consideration of a consumer's immigration status where it could affect the consumer's income or employment. Applies to mortgage originations and certain open-end credit products. Guidance only; no force of law.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2026/06/08/2026-11447/statement-on-ability-to-repay-and-immigration-status</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CFPB</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>FinCEN Advisory FIN-2026-A002: Suspicious Activity Linked to Non-Work-Authorized Workers</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>FinCEN, with FDIC/OCC/NCUA, issued Advisory FIN-2026-A002 directing banks and credit unions to identify and SAR-file transactions tied to payroll fraud schemes involving non-work-authorized workers; $2.5B+ in suspicious activity reported in 2025. Introduces 18 red flags and new SAR key term 'FINANCIALINTEGRITY-2026-A002'.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://home.treasury.gov/news/press-releases/sb0523</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>FinCEN / FDIC / OCC / NCUA</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>California DFPI: Second Modified Proposed Digital Financial Assets Law Regulations</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>California DFPI issued a second modified version of proposed DFAL regulations after OAL disapproval on May 19, 2026. Modifications clarify application (Form MU1), executive officer reporting, and surety bond criteria. DFAL license deadline remains July 1, 2026. Comment period: June 5–22, 2026.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://dfpi.ca.gov/rules-enforcement/laws-and-regulations/digital-financial-assets-law-regulations-opinions-releases/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>CA DFPI</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>NCUA Final Rule: Dependent Care and Board Member Reimbursement</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>NCUA finalized a rule removing prior restrictions on reimbursing FCU volunteer officials for dependent care expenses incurred in connection with board service, reducing barriers to volunteer participation. Effective approximately July 9, 2026. Narrow operational impact for FCUs.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://ncua.gov/newsroom/press-release/2026/ncua-board-approves-final-rule-dependent-care-and-board-member-reimbursement</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>NCUA Q1 2026 Credit Union System Performance Data</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>NCUA released Q1 2026 aggregate data: total assets $2.48T (+4.9% YoY), total loans $1.73T (+4.6% YoY) for federally insured credit unions. Informational; no compliance action required.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://ncua.gov/newsroom/press-release/2026/ncua-releases-first-quarter-2026-credit-union-system-performance-data</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Federal Reserve Governor Barr Speech: Concerns About Weakened Bank Supervision</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Governor Barr at American University raised concerns that simultaneous capital reductions and lighter-touch supervision compound systemic risk; criticized recent CAMELS rating changes as 'grade inflation,' curtailed MRA issuances, and removal of reputation risk. No regulatory effect.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/speech/barr20260606a.htm</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly briefing 2026-06-12 to 2026-06-18
8 items: Joint stablecoin CIP NPRM (Fed/FinCEN/OCC/FDIC/NCUA), SEC Reg NMS
rescission proposal, NACHA Phase 2 ACH fraud monitoring effective, FOMC hawkish
hold, NCUA vital records final rule, three OCC actions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tGfJHqA8qQ6eLKXQXrcSV
</commit_message>
<xml_diff>
--- a/regulatory-changes.xlsx
+++ b/regulatory-changes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2553,6 +2553,286 @@
         <v>2</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Joint NPRM: Customer Identification Program for Payment Stablecoin Issuers (GENIUS Act)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Five federal agencies (Fed, FinCEN, OCC, FDIC, NCUA) jointly proposed a rule requiring permitted payment stablecoin issuers (PPSIs) to maintain customer identification programs comparable to those for banks/credit unions, implementing GENIUS Act AML provisions. CIP obligations limited to direct-to-consumer services. Comments due ~60 days after Federal Register publication (est. mid-August 2026). Banks and CUs with PPSI subsidiaries or stablecoin operations directly affected.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/bcreg20260618a.htm</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Federal Reserve / FinCEN / OCC / FDIC / NCUA</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SEC NPRM: Rescission of Regulation NMS Rules 611 and 610(e)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SEC proposed to rescind Rule 611 (Order Protection / trade-through rule) and Rule 610(e) (prohibition on locked/crossed markets), described as the most significant U.S. equity market structure change in two decades. If adopted, broker-dealers could trade through better-priced exchange quotes. Banks with broker-dealer affiliates or institutional trading operations are directly affected. Comment deadline: August 17, 2026.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/newsroom/press-releases/2026-54-sec-proposes-rescission-regulation-nms-rules-611-610e</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>NACHA Risk Management Phase 2: Universal ACH Fraud Monitoring Effective June 22, 2026</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Phase 2 eliminates all origination-volume thresholds, requiring every RDFI, Originator, Third-Party Sender, and TPSP to implement risk-based processes to detect and prevent fraudulent ACH entries. Effective June 19, 2026 (practical banking-day date June 22, Juneteenth). Completes multi-year rollout begun in Phase 1 (March 2026). All ACH-active banks and credit unions must confirm Phase 2 compliance immediately.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.nacha.org/news/new-nacha-risk-management-rules-now-effect</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>NACHA</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>FOMC Statement: Rates Held at 3.5-3.75%; Hawkish Dot Plot; Warsh Announces Five Task Forces</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>FOMC voted 12-0 to hold the federal funds rate at 3.5-3.75%. June dot plot shifted hawkish: 9 of 18 officials project a 2026 rate hike, median PCE inflation revised to 3.6%. Chair Warsh announced five task forces to overhaul Fed communications, balance sheet management, and the inflation framework. Implementation note effective June 18, 2026.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/newsevents/pressreleases/monetary20260617a.htm</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Federal Reserve</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>NCUA Final Rule: Vital Records Preservation (12 CFR 749)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NCUA updated its 50-year-old catastrophic-act records preservation rule, removing prescriptive Appendices A and B and granting credit unions flexibility in determining vital records preservation log content. Effective July 16, 2026. Credit unions should update records preservation programs before that date. Part of NCUA's deregulation initiative.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://ncua.gov/newsroom/press-release/2026/ncua-board-approves-final-rule-vital-records-preservation</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>NCUA</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>OCC Clarifies Filing Decision Standards (12 CFR 5.13)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>The OCC reaffirmed that all filing decisions are governed by 12 CFR 5.13 and that the agency may approve, conditionally approve, deny, or return as materially deficient any application. No policy change; relevant for institutions planning mergers, acquisitions, de novo applications, or charter conversions.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-47.html</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>OCC Reissues Minority Depository Institution Policy Statement (Bulletin 2026-26)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>OCC reissued its MDI policy statement to align the MDI definition with FIRREA, consistent with EO 14219. Removes references to obsolete agency programs; MDI status preserved for existing designees. Minimal operational impact beyond the 12 OCC-supervised MDIs.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/bulletins/2026/bulletin-2026-26.html</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>OCC June 2026 Enforcement Actions: Two Orders of Prohibition</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Orders of Prohibition against Steven Ho (Quontic Bank, NY) for concealing work with unapproved third-party mortgage brokers, and Danny Seibel (First National Bank of Lindsay, OK) for bank fraud causing insolvency—Seibel pleaded guilty under 18 U.S.C. §1344; bank placed in FDIC receivership October 2024.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.occ.gov/news-issuances/news-releases/2026/nr-occ-2026-48.html</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>